<commit_message>
phoneme stuff pt. :p
</commit_message>
<xml_diff>
--- a/data/phoneme_onset_D/St02_D.xlsx
+++ b/data/phoneme_onset_D/St02_D.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveunibo-my.sharepoint.com/personal/francesca_schiavon10_studio_unibo_it/Documents/Desktop/IMT/TESI/linguistic_pipeline_EEG/data/phoneme_onset_D/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="11_264933A1D3F0523B4FF83E11595ED87656C19017" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A509506D-68A5-4B50-870A-CE41090C1C57}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="11_264933A1D3F0523B4FF83E11595ED87656C19017" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C4D29E28-12D5-4352-A81E-7EA62D76FCF1}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11969" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11971" uniqueCount="395">
   <si>
     <t>BEGIN</t>
   </si>
@@ -1593,7 +1593,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I2397"/>
+  <dimension ref="A1:I2398"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="15.81640625" customWidth="1"/>
@@ -2227,7 +2227,7 @@
         <v>242109</v>
       </c>
       <c r="B28" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C28" t="s">
         <v>46</v>
@@ -5930,7 +5930,7 @@
         <v>836577</v>
       </c>
       <c r="B189" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C189" t="s">
         <v>46</v>
@@ -6022,7 +6022,7 @@
         <v>857745</v>
       </c>
       <c r="B193" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C193" t="s">
         <v>382</v>
@@ -6045,7 +6045,7 @@
         <v>863037</v>
       </c>
       <c r="B194" t="s">
-        <v>65</v>
+        <v>119</v>
       </c>
       <c r="C194" t="s">
         <v>382</v>
@@ -6735,7 +6735,7 @@
         <v>997101</v>
       </c>
       <c r="B224" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="C224" t="s">
         <v>385</v>
@@ -8368,7 +8368,7 @@
         <v>1296981</v>
       </c>
       <c r="B295" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C295" t="s">
         <v>46</v>
@@ -9897,7 +9897,7 @@
         <v>1566873</v>
       </c>
       <c r="B362" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C362" t="s">
         <v>46</v>
@@ -12771,7 +12771,7 @@
         <v>2058588</v>
       </c>
       <c r="B488" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C488" t="s">
         <v>46</v>
@@ -16428,7 +16428,7 @@
         <v>2664522</v>
       </c>
       <c r="B647" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C647" t="s">
         <v>46</v>
@@ -17371,7 +17371,7 @@
         <v>2880612</v>
       </c>
       <c r="B688" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C688" t="s">
         <v>89</v>
@@ -20050,7 +20050,7 @@
         <v>3338370</v>
       </c>
       <c r="B805" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C805" t="s">
         <v>46</v>
@@ -21545,7 +21545,7 @@
         <v>3554460</v>
       </c>
       <c r="B870" t="s">
-        <v>205</v>
+        <v>40</v>
       </c>
       <c r="C870" t="s">
         <v>51</v>
@@ -22212,7 +22212,7 @@
         <v>3676176</v>
       </c>
       <c r="B899" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C899" t="s">
         <v>46</v>
@@ -25593,7 +25593,7 @@
         <v>4311657</v>
       </c>
       <c r="B1046" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C1046" t="s">
         <v>46</v>
@@ -26145,7 +26145,7 @@
         <v>4430727</v>
       </c>
       <c r="B1070" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="C1070" t="s">
         <v>73</v>
@@ -26398,7 +26398,7 @@
         <v>4459392</v>
       </c>
       <c r="B1081" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C1081" t="s">
         <v>46</v>
@@ -29526,7 +29526,7 @@
         <v>4976274</v>
       </c>
       <c r="B1217" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C1217" t="s">
         <v>46</v>
@@ -30733,7 +30733,7 @@
         <v>5191893</v>
       </c>
       <c r="B1270" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C1270" t="s">
         <v>46</v>
@@ -32665,7 +32665,7 @@
         <v>5563656</v>
       </c>
       <c r="B1354" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C1354" t="s">
         <v>261</v>
@@ -35885,7 +35885,7 @@
         <v>6081390</v>
       </c>
       <c r="B1494" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C1494" t="s">
         <v>46</v>
@@ -37541,7 +37541,7 @@
         <v>6362307</v>
       </c>
       <c r="B1566" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C1566" t="s">
         <v>46</v>
@@ -39496,7 +39496,7 @@
         <v>6690411</v>
       </c>
       <c r="B1651" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C1651" t="s">
         <v>46</v>
@@ -47741,7 +47741,7 @@
         <v>8143065</v>
       </c>
       <c r="B2010" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="C2010" t="s">
         <v>346</v>
@@ -47902,7 +47902,7 @@
         <v>8168576</v>
       </c>
       <c r="B2017" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C2017" t="s">
         <v>46</v>
@@ -49512,7 +49512,7 @@
         <v>8483517</v>
       </c>
       <c r="B2087" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C2087" t="s">
         <v>46</v>
@@ -49949,7 +49949,7 @@
         <v>8530263</v>
       </c>
       <c r="B2106" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="C2106" t="s">
         <v>355</v>
@@ -54338,46 +54338,34 @@
       </c>
     </row>
     <row r="2297" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2297">
-        <v>9329796</v>
-      </c>
       <c r="B2297" t="s">
         <v>12</v>
       </c>
       <c r="C2297" t="s">
-        <v>373</v>
-      </c>
-      <c r="D2297" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2297" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2297" t="s">
-        <v>15</v>
+        <v>220</v>
       </c>
       <c r="G2297">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="2298" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2298">
-        <v>9336411</v>
+        <v>9329796</v>
       </c>
       <c r="B2298" t="s">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="C2298" t="s">
         <v>373</v>
       </c>
       <c r="D2298" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="E2298" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F2298" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G2298">
         <v>580</v>
@@ -54385,19 +54373,19 @@
     </row>
     <row r="2299" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2299">
-        <v>9343908</v>
+        <v>9336411</v>
       </c>
       <c r="B2299" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="C2299" t="s">
         <v>373</v>
       </c>
       <c r="D2299" t="s">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="E2299" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F2299" t="s">
         <v>20</v>
@@ -54408,22 +54396,22 @@
     </row>
     <row r="2300" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2300">
-        <v>9346554</v>
+        <v>9343908</v>
       </c>
       <c r="B2300" t="s">
-        <v>42</v>
+        <v>71</v>
       </c>
       <c r="C2300" t="s">
         <v>373</v>
       </c>
       <c r="D2300" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="E2300" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F2300" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2300">
         <v>580</v>
@@ -54431,22 +54419,22 @@
     </row>
     <row r="2301" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2301">
-        <v>9354933</v>
+        <v>9346554</v>
       </c>
       <c r="B2301" t="s">
-        <v>135</v>
+        <v>42</v>
       </c>
       <c r="C2301" t="s">
         <v>373</v>
       </c>
       <c r="D2301" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="E2301" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F2301" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G2301">
         <v>580</v>
@@ -54454,22 +54442,22 @@
     </row>
     <row r="2302" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2302">
-        <v>9361548</v>
+        <v>9354933</v>
       </c>
       <c r="B2302" t="s">
-        <v>12</v>
+        <v>135</v>
       </c>
       <c r="C2302" t="s">
         <v>373</v>
       </c>
       <c r="D2302" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E2302" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F2302" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2302">
         <v>580</v>
@@ -54477,68 +54465,68 @@
     </row>
     <row r="2303" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2303">
-        <v>9390213</v>
+        <v>9361548</v>
       </c>
       <c r="B2303" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="C2303" t="s">
-        <v>31</v>
+        <v>373</v>
       </c>
       <c r="D2303" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="E2303" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="F2303" t="s">
         <v>15</v>
       </c>
       <c r="G2303">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="2304" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2304">
-        <v>9391536</v>
+        <v>9390213</v>
       </c>
       <c r="B2304" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="C2304" t="s">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="D2304" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="E2304" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F2304" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2304">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="2305" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2305">
-        <v>9394182</v>
+        <v>9391536</v>
       </c>
       <c r="B2305" t="s">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="C2305" t="s">
         <v>98</v>
       </c>
       <c r="D2305" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="E2305" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="F2305" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2305">
         <v>582</v>
@@ -54546,45 +54534,45 @@
     </row>
     <row r="2306" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2306">
-        <v>9396387</v>
+        <v>9394182</v>
       </c>
       <c r="B2306" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="C2306" t="s">
-        <v>374</v>
+        <v>98</v>
       </c>
       <c r="D2306" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="E2306" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F2306" t="s">
         <v>15</v>
       </c>
       <c r="G2306">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="2307" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2307">
-        <v>9399915</v>
+        <v>9396387</v>
       </c>
       <c r="B2307" t="s">
-        <v>82</v>
+        <v>12</v>
       </c>
       <c r="C2307" t="s">
         <v>374</v>
       </c>
       <c r="D2307" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="E2307" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="F2307" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G2307">
         <v>583</v>
@@ -54592,22 +54580,22 @@
     </row>
     <row r="2308" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2308">
-        <v>9406971</v>
+        <v>9399915</v>
       </c>
       <c r="B2308" t="s">
-        <v>42</v>
+        <v>82</v>
       </c>
       <c r="C2308" t="s">
         <v>374</v>
       </c>
       <c r="D2308" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="E2308" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="F2308" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2308">
         <v>583</v>
@@ -54615,22 +54603,22 @@
     </row>
     <row r="2309" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2309">
-        <v>9416232</v>
+        <v>9406971</v>
       </c>
       <c r="B2309" t="s">
-        <v>127</v>
+        <v>42</v>
       </c>
       <c r="C2309" t="s">
         <v>374</v>
       </c>
       <c r="D2309" t="s">
-        <v>114</v>
+        <v>32</v>
       </c>
       <c r="E2309" t="s">
-        <v>114</v>
+        <v>26</v>
       </c>
       <c r="F2309" t="s">
-        <v>114</v>
+        <v>15</v>
       </c>
       <c r="G2309">
         <v>583</v>
@@ -54638,22 +54626,22 @@
     </row>
     <row r="2310" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2310">
-        <v>9420201</v>
+        <v>9416232</v>
       </c>
       <c r="B2310" t="s">
-        <v>12</v>
+        <v>127</v>
       </c>
       <c r="C2310" t="s">
         <v>374</v>
       </c>
       <c r="D2310" t="s">
-        <v>13</v>
+        <v>114</v>
       </c>
       <c r="E2310" t="s">
-        <v>14</v>
+        <v>114</v>
       </c>
       <c r="F2310" t="s">
-        <v>15</v>
+        <v>114</v>
       </c>
       <c r="G2310">
         <v>583</v>
@@ -54661,45 +54649,45 @@
     </row>
     <row r="2311" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2311">
-        <v>9432178</v>
+        <v>9420201</v>
       </c>
       <c r="B2311" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C2311" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D2311" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E2311" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F2311" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G2311">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="2312" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2312">
-        <v>9434754</v>
+        <v>9432178</v>
       </c>
       <c r="B2312" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="C2312" t="s">
         <v>375</v>
       </c>
       <c r="D2312" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="E2312" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="F2312" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2312">
         <v>584</v>
@@ -54707,22 +54695,22 @@
     </row>
     <row r="2313" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2313">
-        <v>9436518</v>
+        <v>9434754</v>
       </c>
       <c r="B2313" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="C2313" t="s">
         <v>375</v>
       </c>
       <c r="D2313" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="E2313" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="F2313" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2313">
         <v>584</v>
@@ -54730,22 +54718,22 @@
     </row>
     <row r="2314" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2314">
-        <v>9439164</v>
+        <v>9436518</v>
       </c>
       <c r="B2314" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C2314" t="s">
         <v>375</v>
       </c>
       <c r="D2314" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E2314" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F2314" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2314">
         <v>584</v>
@@ -54753,22 +54741,22 @@
     </row>
     <row r="2315" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2315">
-        <v>9444897</v>
+        <v>9439164</v>
       </c>
       <c r="B2315" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="C2315" t="s">
         <v>375</v>
       </c>
       <c r="D2315" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E2315" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F2315" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2315">
         <v>584</v>
@@ -54776,22 +54764,22 @@
     </row>
     <row r="2316" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2316">
-        <v>9449748</v>
+        <v>9444897</v>
       </c>
       <c r="B2316" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="C2316" t="s">
         <v>375</v>
       </c>
       <c r="D2316" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E2316" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F2316" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="G2316">
         <v>584</v>
@@ -54799,22 +54787,22 @@
     </row>
     <row r="2317" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2317">
-        <v>9451953</v>
+        <v>9449748</v>
       </c>
       <c r="B2317" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="C2317" t="s">
         <v>375</v>
       </c>
       <c r="D2317" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="E2317" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F2317" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2317">
         <v>584</v>
@@ -54822,13 +54810,13 @@
     </row>
     <row r="2318" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2318">
-        <v>9455326</v>
+        <v>9451953</v>
       </c>
       <c r="B2318" t="s">
         <v>12</v>
       </c>
       <c r="C2318" t="s">
-        <v>12</v>
+        <v>375</v>
       </c>
       <c r="D2318" t="s">
         <v>13</v>
@@ -54840,47 +54828,47 @@
         <v>15</v>
       </c>
       <c r="G2318">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="2319" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2319">
-        <v>9457245</v>
+        <v>9455326</v>
       </c>
       <c r="B2319" t="s">
-        <v>119</v>
+        <v>12</v>
       </c>
       <c r="C2319" t="s">
-        <v>376</v>
+        <v>12</v>
       </c>
       <c r="D2319" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="E2319" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F2319" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2319">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="2320" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2320">
-        <v>9461655</v>
+        <v>9457245</v>
       </c>
       <c r="B2320" t="s">
-        <v>59</v>
+        <v>119</v>
       </c>
       <c r="C2320" t="s">
         <v>376</v>
       </c>
       <c r="D2320" t="s">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="E2320" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F2320" t="s">
         <v>11</v>
@@ -54891,22 +54879,22 @@
     </row>
     <row r="2321" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2321">
-        <v>9463419</v>
+        <v>9461655</v>
       </c>
       <c r="B2321" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="C2321" t="s">
         <v>376</v>
       </c>
       <c r="D2321" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="E2321" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="F2321" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2321">
         <v>586</v>
@@ -54914,22 +54902,22 @@
     </row>
     <row r="2322" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2322">
-        <v>9467829</v>
+        <v>9463419</v>
       </c>
       <c r="B2322" t="s">
-        <v>135</v>
+        <v>38</v>
       </c>
       <c r="C2322" t="s">
         <v>376</v>
       </c>
       <c r="D2322" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="E2322" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="F2322" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G2322">
         <v>586</v>
@@ -54937,22 +54925,22 @@
     </row>
     <row r="2323" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2323">
-        <v>9471798</v>
+        <v>9467829</v>
       </c>
       <c r="B2323" t="s">
-        <v>38</v>
+        <v>135</v>
       </c>
       <c r="C2323" t="s">
         <v>376</v>
       </c>
       <c r="D2323" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="E2323" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="F2323" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2323">
         <v>586</v>
@@ -54960,22 +54948,22 @@
     </row>
     <row r="2324" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2324">
-        <v>9475326</v>
+        <v>9471798</v>
       </c>
       <c r="B2324" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C2324" t="s">
         <v>376</v>
       </c>
       <c r="D2324" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="E2324" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="F2324" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2324">
         <v>586</v>
@@ -54983,22 +54971,22 @@
     </row>
     <row r="2325" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2325">
-        <v>9477972</v>
+        <v>9475326</v>
       </c>
       <c r="B2325" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="C2325" t="s">
         <v>376</v>
       </c>
       <c r="D2325" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E2325" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F2325" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2325">
         <v>586</v>
@@ -55006,22 +54994,22 @@
     </row>
     <row r="2326" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2326">
-        <v>9481941</v>
+        <v>9477972</v>
       </c>
       <c r="B2326" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="C2326" t="s">
         <v>376</v>
       </c>
       <c r="D2326" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="E2326" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F2326" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2326">
         <v>586</v>
@@ -55029,16 +55017,16 @@
     </row>
     <row r="2327" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2327">
-        <v>9484176</v>
+        <v>9481941</v>
       </c>
       <c r="B2327" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="C2327" t="s">
         <v>376</v>
       </c>
       <c r="D2327" t="s">
-        <v>9</v>
+        <v>47</v>
       </c>
       <c r="E2327" t="s">
         <v>10</v>
@@ -55052,22 +55040,22 @@
     </row>
     <row r="2328" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2328">
-        <v>9486351</v>
+        <v>9484176</v>
       </c>
       <c r="B2328" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="C2328" t="s">
         <v>376</v>
       </c>
       <c r="D2328" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="E2328" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F2328" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2328">
         <v>586</v>
@@ -55075,45 +55063,45 @@
     </row>
     <row r="2329" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2329">
-        <v>9490320</v>
+        <v>9486351</v>
       </c>
       <c r="B2329" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="C2329" t="s">
-        <v>116</v>
+        <v>376</v>
       </c>
       <c r="D2329" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="E2329" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F2329" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2329">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="2330" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2330">
-        <v>9493248</v>
+        <v>9490320</v>
       </c>
       <c r="B2330" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C2330" t="s">
         <v>116</v>
       </c>
       <c r="D2330" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E2330" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F2330" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2330">
         <v>587</v>
@@ -55121,45 +55109,45 @@
     </row>
     <row r="2331" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2331">
-        <v>9496494</v>
+        <v>9493248</v>
       </c>
       <c r="B2331" t="s">
-        <v>78</v>
+        <v>12</v>
       </c>
       <c r="C2331" t="s">
-        <v>377</v>
+        <v>116</v>
       </c>
       <c r="D2331" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="E2331" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F2331" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2331">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="2332" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2332">
-        <v>9498699</v>
+        <v>9496494</v>
       </c>
       <c r="B2332" t="s">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="C2332" t="s">
         <v>377</v>
       </c>
       <c r="D2332" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="E2332" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F2332" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2332">
         <v>588</v>
@@ -55167,22 +55155,22 @@
     </row>
     <row r="2333" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2333">
-        <v>9503991</v>
+        <v>9498699</v>
       </c>
       <c r="B2333" t="s">
-        <v>68</v>
+        <v>12</v>
       </c>
       <c r="C2333" t="s">
         <v>377</v>
       </c>
       <c r="D2333" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E2333" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F2333" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G2333">
         <v>588</v>
@@ -55190,22 +55178,22 @@
     </row>
     <row r="2334" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2334">
-        <v>9512811</v>
+        <v>9503991</v>
       </c>
       <c r="B2334" t="s">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="C2334" t="s">
         <v>377</v>
       </c>
       <c r="D2334" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E2334" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F2334" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2334">
         <v>588</v>
@@ -55213,45 +55201,45 @@
     </row>
     <row r="2335" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2335">
-        <v>9546207</v>
+        <v>9512811</v>
       </c>
       <c r="B2335" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="C2335" t="s">
-        <v>393</v>
+        <v>377</v>
       </c>
       <c r="D2335" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E2335" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F2335" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G2335">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="2336" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2336">
-        <v>9547650</v>
+        <v>9546207</v>
       </c>
       <c r="B2336" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C2336" t="s">
         <v>393</v>
       </c>
       <c r="D2336" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="E2336" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="F2336" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2336">
         <v>589</v>
@@ -55259,22 +55247,22 @@
     </row>
     <row r="2337" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2337">
-        <v>9552060</v>
+        <v>9547650</v>
       </c>
       <c r="B2337" t="s">
-        <v>135</v>
+        <v>43</v>
       </c>
       <c r="C2337" t="s">
         <v>393</v>
       </c>
       <c r="D2337" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="E2337" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="F2337" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G2337">
         <v>589</v>
@@ -55282,68 +55270,68 @@
     </row>
     <row r="2338" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2338">
-        <v>9553824</v>
+        <v>9552060</v>
       </c>
       <c r="B2338" t="s">
-        <v>12</v>
+        <v>135</v>
       </c>
       <c r="C2338" t="s">
-        <v>12</v>
+        <v>393</v>
       </c>
       <c r="D2338" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E2338" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F2338" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2338">
-        <v>590</v>
+        <v>589</v>
       </c>
     </row>
     <row r="2339" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2339">
-        <v>9556487</v>
+        <v>9553824</v>
       </c>
       <c r="B2339" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="C2339" t="s">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="D2339" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="E2339" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="F2339" t="s">
         <v>15</v>
       </c>
       <c r="G2339">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="2340" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2340">
-        <v>9558234</v>
+        <v>9556487</v>
       </c>
       <c r="B2340" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C2340" t="s">
         <v>51</v>
       </c>
       <c r="D2340" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E2340" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="F2340" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2340">
         <v>591</v>
@@ -55351,92 +55339,92 @@
     </row>
     <row r="2341" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2341">
-        <v>9560439</v>
+        <v>9558234</v>
       </c>
       <c r="B2341" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C2341" t="s">
-        <v>394</v>
+        <v>51</v>
       </c>
       <c r="D2341" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E2341" t="s">
         <v>10</v>
       </c>
       <c r="F2341" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="G2341">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="2342" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2342">
-        <v>9561762</v>
+        <v>9560439</v>
       </c>
       <c r="B2342" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C2342" t="s">
         <v>394</v>
       </c>
       <c r="D2342" t="s">
-        <v>47</v>
+        <v>18</v>
       </c>
       <c r="E2342" t="s">
         <v>10</v>
       </c>
       <c r="F2342" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="G2342">
         <v>592</v>
       </c>
-      <c r="I2342" s="2"/>
     </row>
     <row r="2343" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2343">
-        <v>9563085</v>
+        <v>9561762</v>
       </c>
       <c r="B2343" t="s">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="C2343" t="s">
         <v>394</v>
       </c>
       <c r="D2343" t="s">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="E2343" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F2343" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2343">
         <v>592</v>
       </c>
+      <c r="I2343" s="2"/>
     </row>
     <row r="2344" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2344">
-        <v>9566613</v>
+        <v>9563085</v>
       </c>
       <c r="B2344" t="s">
-        <v>135</v>
+        <v>12</v>
       </c>
       <c r="C2344" t="s">
         <v>394</v>
       </c>
       <c r="D2344" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E2344" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F2344" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G2344">
         <v>592</v>
@@ -55444,22 +55432,22 @@
     </row>
     <row r="2345" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2345">
-        <v>9571023</v>
+        <v>9566613</v>
       </c>
       <c r="B2345" t="s">
-        <v>38</v>
+        <v>135</v>
       </c>
       <c r="C2345" t="s">
         <v>394</v>
       </c>
       <c r="D2345" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="E2345" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="F2345" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2345">
         <v>592</v>
@@ -55467,45 +55455,45 @@
     </row>
     <row r="2346" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2346">
-        <v>9573228</v>
+        <v>9571023</v>
       </c>
       <c r="B2346" t="s">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="C2346" t="s">
-        <v>174</v>
+        <v>394</v>
       </c>
       <c r="D2346" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="E2346" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="F2346" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G2346">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="2347" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2347">
-        <v>9577197</v>
+        <v>9573228</v>
       </c>
       <c r="B2347" t="s">
-        <v>24</v>
+        <v>65</v>
       </c>
       <c r="C2347" t="s">
         <v>174</v>
       </c>
       <c r="D2347" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="E2347" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F2347" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2347">
         <v>593</v>
@@ -55513,45 +55501,45 @@
     </row>
     <row r="2348" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2348">
-        <v>9581166</v>
+        <v>9577197</v>
       </c>
       <c r="B2348" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="C2348" t="s">
-        <v>378</v>
+        <v>174</v>
       </c>
       <c r="D2348" t="s">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="E2348" t="s">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="F2348" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G2348">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="2349" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2349">
-        <v>9583812</v>
+        <v>9581166</v>
       </c>
       <c r="B2349" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="C2349" t="s">
         <v>378</v>
       </c>
       <c r="D2349" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="E2349" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="F2349" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2349">
         <v>594</v>
@@ -55559,22 +55547,22 @@
     </row>
     <row r="2350" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2350">
-        <v>9585135</v>
+        <v>9583812</v>
       </c>
       <c r="B2350" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="C2350" t="s">
         <v>378</v>
       </c>
       <c r="D2350" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="E2350" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F2350" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2350">
         <v>594</v>
@@ -55582,19 +55570,19 @@
     </row>
     <row r="2351" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2351">
-        <v>9589986</v>
+        <v>9585135</v>
       </c>
       <c r="B2351" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="C2351" t="s">
         <v>378</v>
       </c>
       <c r="D2351" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="E2351" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F2351" t="s">
         <v>11</v>
@@ -55605,22 +55593,22 @@
     </row>
     <row r="2352" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2352">
-        <v>9594837</v>
+        <v>9589986</v>
       </c>
       <c r="B2352" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="C2352" t="s">
         <v>378</v>
       </c>
       <c r="D2352" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E2352" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F2352" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2352">
         <v>594</v>
@@ -55628,45 +55616,45 @@
     </row>
     <row r="2353" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2353">
-        <v>9596601</v>
+        <v>9594837</v>
       </c>
       <c r="B2353" t="s">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="C2353" t="s">
-        <v>57</v>
+        <v>378</v>
       </c>
       <c r="D2353" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E2353" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F2353" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2353">
-        <v>595</v>
+        <v>594</v>
       </c>
     </row>
     <row r="2354" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2354">
-        <v>9598365</v>
+        <v>9596601</v>
       </c>
       <c r="B2354" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="C2354" t="s">
         <v>57</v>
       </c>
       <c r="D2354" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="E2354" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F2354" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2354">
         <v>595</v>
@@ -55674,45 +55662,45 @@
     </row>
     <row r="2355" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2355">
-        <v>9601452</v>
+        <v>9598365</v>
       </c>
       <c r="B2355" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C2355" t="s">
-        <v>379</v>
+        <v>57</v>
       </c>
       <c r="D2355" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="E2355" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F2355" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G2355">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="2356" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2356">
-        <v>9603657</v>
+        <v>9601452</v>
       </c>
       <c r="B2356" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C2356" t="s">
         <v>379</v>
       </c>
       <c r="D2356" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E2356" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F2356" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2356">
         <v>596</v>
@@ -55720,22 +55708,22 @@
     </row>
     <row r="2357" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2357">
-        <v>9607626</v>
+        <v>9603657</v>
       </c>
       <c r="B2357" t="s">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="C2357" t="s">
         <v>379</v>
       </c>
       <c r="D2357" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="E2357" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F2357" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G2357">
         <v>596</v>
@@ -55743,19 +55731,19 @@
     </row>
     <row r="2358" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2358">
-        <v>9612036</v>
+        <v>9607626</v>
       </c>
       <c r="B2358" t="s">
-        <v>16</v>
+        <v>65</v>
       </c>
       <c r="C2358" t="s">
         <v>379</v>
       </c>
       <c r="D2358" t="s">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="E2358" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F2358" t="s">
         <v>20</v>
@@ -55766,22 +55754,22 @@
     </row>
     <row r="2359" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2359">
-        <v>9614241</v>
+        <v>9612036</v>
       </c>
       <c r="B2359" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C2359" t="s">
         <v>379</v>
       </c>
       <c r="D2359" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E2359" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F2359" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2359">
         <v>596</v>
@@ -55789,22 +55777,22 @@
     </row>
     <row r="2360" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2360">
-        <v>9616887</v>
+        <v>9614241</v>
       </c>
       <c r="B2360" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="C2360" t="s">
         <v>379</v>
       </c>
       <c r="D2360" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="E2360" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F2360" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2360">
         <v>596</v>
@@ -55812,22 +55800,22 @@
     </row>
     <row r="2361" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2361">
-        <v>9618210</v>
+        <v>9616887</v>
       </c>
       <c r="B2361" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C2361" t="s">
         <v>379</v>
       </c>
       <c r="D2361" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E2361" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="F2361" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2361">
         <v>596</v>
@@ -55835,45 +55823,45 @@
     </row>
     <row r="2362" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2362">
-        <v>9620415</v>
+        <v>9618210</v>
       </c>
       <c r="B2362" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="C2362" t="s">
-        <v>160</v>
+        <v>379</v>
       </c>
       <c r="D2362" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="E2362" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="F2362" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2362">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="2363" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2363">
-        <v>9622179</v>
+        <v>9620415</v>
       </c>
       <c r="B2363" t="s">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="C2363" t="s">
         <v>160</v>
       </c>
       <c r="D2363" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="E2363" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F2363" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2363">
         <v>597</v>
@@ -55881,42 +55869,42 @@
     </row>
     <row r="2364" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2364">
-        <v>9625266</v>
+        <v>9622179</v>
       </c>
       <c r="B2364" t="s">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="C2364" t="s">
-        <v>380</v>
+        <v>160</v>
       </c>
       <c r="D2364" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="E2364" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F2364" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2364">
-        <v>598</v>
+        <v>597</v>
       </c>
     </row>
     <row r="2365" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2365">
-        <v>9626589</v>
+        <v>9625266</v>
       </c>
       <c r="B2365" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C2365" t="s">
         <v>380</v>
       </c>
       <c r="D2365" t="s">
-        <v>47</v>
+        <v>18</v>
       </c>
       <c r="E2365" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F2365" t="s">
         <v>11</v>
@@ -55927,22 +55915,22 @@
     </row>
     <row r="2366" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2366">
-        <v>9629235</v>
+        <v>9626589</v>
       </c>
       <c r="B2366" t="s">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="C2366" t="s">
         <v>380</v>
       </c>
       <c r="D2366" t="s">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="E2366" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F2366" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2366">
         <v>598</v>
@@ -55950,22 +55938,22 @@
     </row>
     <row r="2367" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2367">
-        <v>9635409</v>
+        <v>9629235</v>
       </c>
       <c r="B2367" t="s">
-        <v>83</v>
+        <v>12</v>
       </c>
       <c r="C2367" t="s">
         <v>380</v>
       </c>
       <c r="D2367" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="E2367" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F2367" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G2367">
         <v>598</v>
@@ -55973,22 +55961,22 @@
     </row>
     <row r="2368" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2368">
-        <v>9642906</v>
+        <v>9635409</v>
       </c>
       <c r="B2368" t="s">
-        <v>12</v>
+        <v>83</v>
       </c>
       <c r="C2368" t="s">
         <v>380</v>
       </c>
       <c r="D2368" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="E2368" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F2368" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2368">
         <v>598</v>
@@ -55996,68 +55984,68 @@
     </row>
     <row r="2369" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2369">
-        <v>9665397</v>
+        <v>9642906</v>
       </c>
       <c r="B2369" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C2369" t="s">
-        <v>56</v>
+        <v>380</v>
       </c>
       <c r="D2369" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E2369" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F2369" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2369">
-        <v>599</v>
+        <v>598</v>
       </c>
     </row>
     <row r="2370" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2370">
-        <v>9668179</v>
+        <v>9665397</v>
       </c>
       <c r="B2370" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="C2370" t="s">
-        <v>189</v>
+        <v>56</v>
       </c>
       <c r="D2370" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="E2370" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F2370" t="s">
         <v>11</v>
       </c>
       <c r="G2370">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="2371" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2371">
-        <v>9669630</v>
+        <v>9668179</v>
       </c>
       <c r="B2371" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C2371" t="s">
         <v>189</v>
       </c>
       <c r="D2371" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E2371" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="F2371" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2371">
         <v>600</v>
@@ -56065,22 +56053,22 @@
     </row>
     <row r="2372" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2372">
-        <v>9671130</v>
+        <v>9669630</v>
       </c>
       <c r="B2372" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="C2372" t="s">
         <v>189</v>
       </c>
       <c r="D2372" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="E2372" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="F2372" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2372">
         <v>600</v>
@@ -56088,22 +56076,22 @@
     </row>
     <row r="2373" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2373">
-        <v>9673776</v>
+        <v>9671130</v>
       </c>
       <c r="B2373" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="C2373" t="s">
         <v>189</v>
       </c>
       <c r="D2373" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E2373" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="F2373" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2373">
         <v>600</v>
@@ -56111,45 +56099,45 @@
     </row>
     <row r="2374" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2374">
-        <v>9676863</v>
+        <v>9673776</v>
       </c>
       <c r="B2374" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="C2374" t="s">
-        <v>39</v>
+        <v>189</v>
       </c>
       <c r="D2374" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="E2374" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="F2374" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G2374">
-        <v>601</v>
+        <v>600</v>
       </c>
     </row>
     <row r="2375" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2375">
-        <v>9679950</v>
+        <v>9676863</v>
       </c>
       <c r="B2375" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="C2375" t="s">
         <v>39</v>
       </c>
       <c r="D2375" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="E2375" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="F2375" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2375">
         <v>601</v>
@@ -56157,22 +56145,22 @@
     </row>
     <row r="2376" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2376">
-        <v>9682155</v>
+        <v>9679950</v>
       </c>
       <c r="B2376" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C2376" t="s">
         <v>39</v>
       </c>
       <c r="D2376" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="E2376" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="F2376" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2376">
         <v>601</v>
@@ -56180,22 +56168,22 @@
     </row>
     <row r="2377" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2377">
-        <v>9685683</v>
+        <v>9682155</v>
       </c>
       <c r="B2377" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C2377" t="s">
         <v>39</v>
       </c>
       <c r="D2377" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E2377" t="s">
         <v>10</v>
       </c>
       <c r="F2377" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="G2377">
         <v>601</v>
@@ -56203,22 +56191,22 @@
     </row>
     <row r="2378" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2378">
-        <v>9690093</v>
+        <v>9685683</v>
       </c>
       <c r="B2378" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C2378" t="s">
         <v>39</v>
       </c>
       <c r="D2378" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="E2378" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F2378" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2378">
         <v>601</v>
@@ -56226,22 +56214,22 @@
     </row>
     <row r="2379" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2379">
-        <v>9696708</v>
+        <v>9690093</v>
       </c>
       <c r="B2379" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C2379" t="s">
         <v>39</v>
       </c>
       <c r="D2379" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="E2379" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F2379" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2379">
         <v>601</v>
@@ -56249,22 +56237,22 @@
     </row>
     <row r="2380" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2380">
-        <v>9700236</v>
+        <v>9696708</v>
       </c>
       <c r="B2380" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C2380" t="s">
         <v>39</v>
       </c>
       <c r="D2380" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E2380" t="s">
         <v>10</v>
       </c>
       <c r="F2380" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="G2380">
         <v>601</v>
@@ -56272,22 +56260,22 @@
     </row>
     <row r="2381" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2381">
-        <v>9703323</v>
+        <v>9700236</v>
       </c>
       <c r="B2381" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C2381" t="s">
         <v>39</v>
       </c>
       <c r="D2381" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="E2381" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="F2381" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2381">
         <v>601</v>
@@ -56295,45 +56283,45 @@
     </row>
     <row r="2382" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2382">
-        <v>9713907</v>
+        <v>9703323</v>
       </c>
       <c r="B2382" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C2382" t="s">
-        <v>102</v>
+        <v>39</v>
       </c>
       <c r="D2382" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="E2382" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="F2382" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2382">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="2383" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2383">
-        <v>9715150</v>
+        <v>9713907</v>
       </c>
       <c r="B2383" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C2383" t="s">
         <v>102</v>
       </c>
       <c r="D2383" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E2383" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="F2383" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2383">
         <v>602</v>
@@ -56341,22 +56329,22 @@
     </row>
     <row r="2384" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2384">
-        <v>9717721</v>
+        <v>9715150</v>
       </c>
       <c r="B2384" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C2384" t="s">
         <v>102</v>
       </c>
       <c r="D2384" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="E2384" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="F2384" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2384">
         <v>602</v>
@@ -56364,45 +56352,45 @@
     </row>
     <row r="2385" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2385">
-        <v>9719481</v>
+        <v>9717721</v>
       </c>
       <c r="B2385" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="C2385" t="s">
-        <v>48</v>
+        <v>102</v>
       </c>
       <c r="D2385" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E2385" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F2385" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2385">
-        <v>603</v>
+        <v>602</v>
       </c>
     </row>
     <row r="2386" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2386">
-        <v>9723168</v>
+        <v>9719481</v>
       </c>
       <c r="B2386" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C2386" t="s">
         <v>48</v>
       </c>
       <c r="D2386" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="E2386" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="F2386" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2386">
         <v>603</v>
@@ -56410,22 +56398,22 @@
     </row>
     <row r="2387" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2387">
-        <v>9724932</v>
+        <v>9723168</v>
       </c>
       <c r="B2387" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="C2387" t="s">
         <v>48</v>
       </c>
       <c r="D2387" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="E2387" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="F2387" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2387">
         <v>603</v>
@@ -56433,22 +56421,22 @@
     </row>
     <row r="2388" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2388">
-        <v>9730665</v>
+        <v>9724932</v>
       </c>
       <c r="B2388" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="C2388" t="s">
         <v>48</v>
       </c>
       <c r="D2388" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="E2388" t="s">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="F2388" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2388">
         <v>603</v>
@@ -56456,22 +56444,22 @@
     </row>
     <row r="2389" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2389">
-        <v>9732521</v>
+        <v>9730665</v>
       </c>
       <c r="B2389" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C2389" t="s">
         <v>48</v>
       </c>
       <c r="D2389" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="E2389" t="s">
-        <v>14</v>
+        <v>50</v>
       </c>
       <c r="F2389" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2389">
         <v>603</v>
@@ -56479,45 +56467,45 @@
     </row>
     <row r="2390" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2390">
-        <v>9735075</v>
+        <v>9732521</v>
       </c>
       <c r="B2390" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C2390" t="s">
-        <v>116</v>
+        <v>48</v>
       </c>
       <c r="D2390" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E2390" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F2390" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2390">
-        <v>604</v>
+        <v>603</v>
       </c>
     </row>
     <row r="2391" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2391">
-        <v>9737055</v>
+        <v>9735075</v>
       </c>
       <c r="B2391" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C2391" t="s">
         <v>116</v>
       </c>
       <c r="D2391" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E2391" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F2391" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2391">
         <v>604</v>
@@ -56525,45 +56513,45 @@
     </row>
     <row r="2392" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2392">
-        <v>9740808</v>
+        <v>9737055</v>
       </c>
       <c r="B2392" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C2392" t="s">
-        <v>17</v>
+        <v>116</v>
       </c>
       <c r="D2392" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E2392" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F2392" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G2392">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
     <row r="2393" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2393">
-        <v>9743895</v>
+        <v>9740808</v>
       </c>
       <c r="B2393" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C2393" t="s">
         <v>17</v>
       </c>
       <c r="D2393" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E2393" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F2393" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2393">
         <v>605</v>
@@ -56571,22 +56559,22 @@
     </row>
     <row r="2394" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2394">
-        <v>9746541</v>
+        <v>9743895</v>
       </c>
       <c r="B2394" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="C2394" t="s">
         <v>17</v>
       </c>
       <c r="D2394" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="E2394" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F2394" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2394">
         <v>605</v>
@@ -56594,22 +56582,22 @@
     </row>
     <row r="2395" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2395">
-        <v>9748746</v>
+        <v>9746541</v>
       </c>
       <c r="B2395" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C2395" t="s">
         <v>17</v>
       </c>
       <c r="D2395" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E2395" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F2395" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2395">
         <v>605</v>
@@ -56617,22 +56605,22 @@
     </row>
     <row r="2396" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2396">
-        <v>9755361</v>
+        <v>9748746</v>
       </c>
       <c r="B2396" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C2396" t="s">
         <v>17</v>
       </c>
       <c r="D2396" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E2396" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F2396" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G2396">
         <v>605</v>
@@ -56640,24 +56628,47 @@
     </row>
     <row r="2397" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2397">
-        <v>9759771</v>
+        <v>9755361</v>
       </c>
       <c r="B2397" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="C2397" t="s">
         <v>17</v>
       </c>
       <c r="D2397" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2397" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2397" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2397">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="2398" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2398">
+        <v>9759771</v>
+      </c>
+      <c r="B2398" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2398" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2398" t="s">
         <v>13</v>
       </c>
-      <c r="E2397" t="s">
+      <c r="E2398" t="s">
         <v>14</v>
       </c>
-      <c r="F2397" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2397">
+      <c r="F2398" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2398">
         <v>605</v>
       </c>
     </row>

</xml_diff>